<commit_message>
Updated app.py with predictive analytics
</commit_message>
<xml_diff>
--- a/Data/complaints_db.xlsx
+++ b/Data/complaints_db.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H159"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6767,7 +6767,87 @@
         </is>
       </c>
       <c r="H159" s="2" t="n">
-        <v>45915.91527263559</v>
+        <v>45915.91527263889</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>C159</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>U006</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>P007</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>V007</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>packaging issue</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="n">
+        <v>45916.6733633449</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>C160</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>U007</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>P004</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>V004</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>bad product</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="n">
+        <v>45916.67621063657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>